<commit_message>
G - Renamed ASVS Sprint 1 and updated ASVS Sprint 2
</commit_message>
<xml_diff>
--- a/Derivables/Sprint2/ASVS_5.0_Tracker_Kryptos.xlsx
+++ b/Derivables/Sprint2/ASVS_5.0_Tracker_Kryptos.xlsx
@@ -1746,34 +1746,34 @@
         <v>8</v>
       </c>
       <c r="D6" s="4" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="E6" s="5" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="F6" s="4" t="n">
         <v>19</v>
       </c>
       <c r="G6" s="4" t="n">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="H6" s="5" t="n">
-        <v>0</v>
+        <v>0.5789473684210527</v>
       </c>
       <c r="I6" s="4" t="n">
         <v>3</v>
       </c>
       <c r="J6" s="4" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K6" s="5" t="n">
-        <v>0</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="L6" s="4" t="n">
-        <v>0</v>
+        <v>17</v>
       </c>
       <c r="M6" s="5" t="n">
-        <v>0</v>
+        <v>0.5666666666666667</v>
       </c>
     </row>
     <row r="7" ht="18" customHeight="1">
@@ -1789,10 +1789,10 @@
         <v>4</v>
       </c>
       <c r="D7" s="7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E7" s="8" t="n">
-        <v>0.5</v>
+        <v>0.75</v>
       </c>
       <c r="F7" s="7" t="n">
         <v>7</v>
@@ -1807,16 +1807,16 @@
         <v>2</v>
       </c>
       <c r="J7" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K7" s="8" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="L7" s="7" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="M7" s="8" t="n">
-        <v>0.3846153846153846</v>
+        <v>0.5384615384615384</v>
       </c>
     </row>
     <row r="8" ht="18" customHeight="1">
@@ -1884,25 +1884,25 @@
         <v>8</v>
       </c>
       <c r="G9" s="7" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H9" s="8" t="n">
-        <v>0</v>
+        <v>0.25</v>
       </c>
       <c r="I9" s="7" t="n">
         <v>6</v>
       </c>
       <c r="J9" s="7" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="K9" s="8" t="n">
-        <v>0</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="L9" s="7" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="M9" s="8" t="n">
-        <v>0.0625</v>
+        <v>0.4375</v>
       </c>
     </row>
     <row r="10" ht="18" customHeight="1">
@@ -1927,25 +1927,25 @@
         <v>5</v>
       </c>
       <c r="G10" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H10" s="5" t="n">
-        <v>0.4</v>
+        <v>0.6</v>
       </c>
       <c r="I10" s="4" t="n">
         <v>4</v>
       </c>
       <c r="J10" s="4" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="K10" s="5" t="n">
-        <v>0</v>
+        <v>0.75</v>
       </c>
       <c r="L10" s="4" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="M10" s="5" t="n">
-        <v>0.4615384615384616</v>
+        <v>0.7692307692307693</v>
       </c>
     </row>
     <row r="11" ht="18" customHeight="1">
@@ -1961,19 +1961,19 @@
         <v>13</v>
       </c>
       <c r="D11" s="7" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="E11" s="8" t="n">
-        <v>0.3846153846153846</v>
+        <v>0.5384615384615384</v>
       </c>
       <c r="F11" s="7" t="n">
         <v>22</v>
       </c>
       <c r="G11" s="7" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H11" s="8" t="n">
-        <v>0.09090909090909091</v>
+        <v>0.1818181818181818</v>
       </c>
       <c r="I11" s="7" t="n">
         <v>12</v>
@@ -1985,10 +1985,10 @@
         <v>0</v>
       </c>
       <c r="L11" s="7" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="M11" s="8" t="n">
-        <v>0.148936170212766</v>
+        <v>0.2340425531914894</v>
       </c>
     </row>
     <row r="12" ht="18" customHeight="1">
@@ -2004,19 +2004,19 @@
         <v>6</v>
       </c>
       <c r="D12" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E12" s="5" t="n">
-        <v>0.3333333333333333</v>
+        <v>0.5</v>
       </c>
       <c r="F12" s="4" t="n">
         <v>12</v>
       </c>
       <c r="G12" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H12" s="5" t="n">
-        <v>0.1666666666666667</v>
+        <v>0.25</v>
       </c>
       <c r="I12" s="4" t="n">
         <v>1</v>
@@ -2028,10 +2028,10 @@
         <v>0</v>
       </c>
       <c r="L12" s="4" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="M12" s="5" t="n">
-        <v>0.2105263157894737</v>
+        <v>0.3157894736842105</v>
       </c>
     </row>
     <row r="13" ht="18" customHeight="1">
@@ -2065,16 +2065,16 @@
         <v>6</v>
       </c>
       <c r="J13" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K13" s="8" t="n">
-        <v>0</v>
+        <v>0.1666666666666667</v>
       </c>
       <c r="L13" s="7" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M13" s="8" t="n">
-        <v>0.2307692307692308</v>
+        <v>0.3076923076923077</v>
       </c>
     </row>
     <row r="14" ht="18" customHeight="1">
@@ -2099,10 +2099,10 @@
         <v>3</v>
       </c>
       <c r="G14" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H14" s="5" t="n">
-        <v>0</v>
+        <v>0.3333333333333333</v>
       </c>
       <c r="I14" s="4" t="n">
         <v>0</v>
@@ -2114,10 +2114,10 @@
         <v>0</v>
       </c>
       <c r="L14" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M14" s="5" t="n">
-        <v>0.5714285714285714</v>
+        <v>0.7142857142857143</v>
       </c>
     </row>
     <row r="15" ht="18" customHeight="1">
@@ -2133,19 +2133,19 @@
         <v>5</v>
       </c>
       <c r="D15" s="7" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E15" s="8" t="n">
-        <v>0</v>
+        <v>0.4</v>
       </c>
       <c r="F15" s="7" t="n">
         <v>24</v>
       </c>
       <c r="G15" s="7" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H15" s="8" t="n">
-        <v>0</v>
+        <v>0.125</v>
       </c>
       <c r="I15" s="7" t="n">
         <v>7</v>
@@ -2157,10 +2157,10 @@
         <v>0</v>
       </c>
       <c r="L15" s="7" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="M15" s="8" t="n">
-        <v>0</v>
+        <v>0.1388888888888889</v>
       </c>
     </row>
     <row r="16" ht="18" customHeight="1">
@@ -2185,25 +2185,25 @@
         <v>11</v>
       </c>
       <c r="G16" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H16" s="5" t="n">
-        <v>0.5454545454545454</v>
+        <v>0.6363636363636364</v>
       </c>
       <c r="I16" s="4" t="n">
         <v>10</v>
       </c>
       <c r="J16" s="4" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="K16" s="5" t="n">
-        <v>0.1</v>
+        <v>0.6</v>
       </c>
       <c r="L16" s="4" t="n">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="M16" s="5" t="n">
-        <v>0.4166666666666667</v>
+        <v>0.6666666666666666</v>
       </c>
     </row>
     <row r="17" ht="18" customHeight="1">
@@ -2262,34 +2262,34 @@
         <v>1</v>
       </c>
       <c r="D18" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E18" s="5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F18" s="4" t="n">
         <v>12</v>
       </c>
       <c r="G18" s="4" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="H18" s="5" t="n">
-        <v>0.25</v>
+        <v>0.75</v>
       </c>
       <c r="I18" s="4" t="n">
         <v>8</v>
       </c>
       <c r="J18" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K18" s="5" t="n">
-        <v>0.125</v>
+        <v>0.25</v>
       </c>
       <c r="L18" s="4" t="n">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="M18" s="5" t="n">
-        <v>0.1904761904761905</v>
+        <v>0.5714285714285714</v>
       </c>
     </row>
     <row r="19" ht="18" customHeight="1">
@@ -2357,25 +2357,25 @@
         <v>10</v>
       </c>
       <c r="G20" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H20" s="5" t="n">
-        <v>0.1</v>
+        <v>0.3</v>
       </c>
       <c r="I20" s="4" t="n">
         <v>8</v>
       </c>
       <c r="J20" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K20" s="5" t="n">
-        <v>0</v>
+        <v>0.125</v>
       </c>
       <c r="L20" s="4" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="M20" s="5" t="n">
-        <v>0.09523809523809523</v>
+        <v>0.2380952380952381</v>
       </c>
     </row>
     <row r="21" ht="18" customHeight="1">
@@ -2487,34 +2487,34 @@
         <v>70</v>
       </c>
       <c r="D23" s="10" t="n">
-        <v>24</v>
+        <v>35</v>
       </c>
       <c r="E23" s="11" t="n">
-        <v>0.3428571428571429</v>
+        <v>0.5</v>
       </c>
       <c r="F23" s="10" t="n">
         <v>183</v>
       </c>
       <c r="G23" s="10" t="n">
-        <v>23</v>
+        <v>53</v>
       </c>
       <c r="H23" s="11" t="n">
-        <v>0.1256830601092896</v>
+        <v>0.2896174863387978</v>
       </c>
       <c r="I23" s="10" t="n">
         <v>92</v>
       </c>
       <c r="J23" s="10" t="n">
-        <v>2</v>
+        <v>20</v>
       </c>
       <c r="K23" s="11" t="n">
-        <v>0.02173913043478261</v>
+        <v>0.2173913043478261</v>
       </c>
       <c r="L23" s="10" t="n">
-        <v>49</v>
+        <v>108</v>
       </c>
       <c r="M23" s="11" t="n">
-        <v>0.1420289855072464</v>
+        <v>0.3130434782608696</v>
       </c>
     </row>
   </sheetData>
@@ -2860,15 +2860,19 @@
       </c>
       <c r="F8" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G8" s="21" t="inlineStr">
         <is>
-          <t>Applicable to Kryptos due to the need to distinguish access tokens from refresh tokens so that each is accepted only for its intended purpose.</t>
-        </is>
-      </c>
-      <c r="H8" s="21" t="n"/>
+          <t>Only one JWT type is issued (an access token with sub + role + iat + exp). There is no separate ID / refresh / authorization token to mis-route, so token-type confusion is not exposed.</t>
+        </is>
+      </c>
+      <c r="H8" s="21" t="inlineStr">
+        <is>
+          <t>JwtService.generateToken</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="37" customHeight="1">
       <c r="A9" s="14" t="inlineStr">
@@ -2896,15 +2900,19 @@
       </c>
       <c r="F9" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="G9" s="16" t="inlineStr">
         <is>
-          <t>Applicable to Kryptos due to the need to accept only tokens whose aud claim targets the Kryptos API.</t>
-        </is>
-      </c>
-      <c r="H9" s="16" t="n"/>
+          <t>JWTs are currently issued without an audience (aud) claim. Adding aud=kryptos at sign time and validating it at verify time is a small, low-risk change targeted for Sprint 3.</t>
+        </is>
+      </c>
+      <c r="H9" s="16" t="inlineStr">
+        <is>
+          <t>JwtService.generateToken / extractAllClaims</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="30" customHeight="1">
       <c r="A10" s="19" t="inlineStr">
@@ -3294,15 +3302,19 @@
       </c>
       <c r="F11" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G11" s="26" t="inlineStr">
         <is>
-          <t>Applicable to Kryptos due to the use of JWT claims for authorization decisions.</t>
-        </is>
-      </c>
-      <c r="H11" s="21" t="n"/>
+          <t>Authorization decisions are derived from the role claim in the JWT (used by the @PreAuthorize hasRole(...) checks via Spring Security). The resource server enforces these decisions on every request through JwtAuthFilter + GlobalMethodSecurity.</t>
+        </is>
+      </c>
+      <c r="H11" s="21" t="inlineStr">
+        <is>
+          <t>JwtAuthFilter.java; SecurityConfig#@EnableMethodSecurity</t>
+        </is>
+      </c>
     </row>
     <row r="12" hidden="1" ht="64" customHeight="1">
       <c r="A12" s="14" t="inlineStr">
@@ -3508,15 +3520,19 @@
       </c>
       <c r="F18" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G18" s="16" t="inlineStr">
         <is>
-          <t>Applicable to Kryptos due to the presence of short-lived activation and password-reset codes.</t>
-        </is>
-      </c>
-      <c r="H18" s="16" t="n"/>
+          <t>Kryptos does not implement an OAuth authorization code flow. No authorization code is issued, so the maximum-lifetime requirement has no surface to violate.</t>
+        </is>
+      </c>
+      <c r="H18" s="16" t="inlineStr">
+        <is>
+          <t>No OAuth in backend/pom.xml or backend/src/main</t>
+        </is>
+      </c>
     </row>
     <row r="19" hidden="1" ht="30" customHeight="1">
       <c r="A19" s="19" t="inlineStr">
@@ -3576,15 +3592,19 @@
       </c>
       <c r="F20" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G20" s="16" t="inlineStr">
         <is>
-          <t>Applicable to Kryptos due to the use of refresh tokens that must resist replay.</t>
-        </is>
-      </c>
-      <c r="H20" s="16" t="n"/>
+          <t>Kryptos does not issue refresh tokens. There is no refresh-token replay surface to mitigate.</t>
+        </is>
+      </c>
+      <c r="H20" s="16" t="inlineStr">
+        <is>
+          <t>JwtService.generateToken (single access-token issuance only)</t>
+        </is>
+      </c>
     </row>
     <row r="21" hidden="1" ht="30" customHeight="1">
       <c r="A21" s="19" t="inlineStr">
@@ -3676,15 +3696,19 @@
       </c>
       <c r="F23" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G23" s="21" t="inlineStr">
         <is>
-          <t>Applicable to Kryptos due to the long-lived nature of refresh tokens requiring an absolute expiration.</t>
-        </is>
-      </c>
-      <c r="H23" s="21" t="n"/>
+          <t>Kryptos does not issue refresh tokens (see V10.4.5). Access tokens have an absolute expiration (exp claim, default 1 h), enforced on every request.</t>
+        </is>
+      </c>
+      <c r="H23" s="21" t="inlineStr">
+        <is>
+          <t>JwtService.isTokenExpired</t>
+        </is>
+      </c>
     </row>
     <row r="24" ht="46" customHeight="1">
       <c r="A24" s="14" t="inlineStr">
@@ -3712,16 +3736,19 @@
       </c>
       <c r="F24" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G24" s="16" t="inlineStr">
         <is>
-          <t xml:space="preserve">Applicable to Kryptos due to the need to revoke active tokens through administrative actions.
-</t>
-        </is>
-      </c>
-      <c r="H24" s="16" t="n"/>
+          <t>Kryptos does not issue refresh tokens or opaque reference access tokens; access tokens are self-contained JWTs that simply expire. There is no revocable token-store surface in scope.</t>
+        </is>
+      </c>
+      <c r="H24" s="16" t="inlineStr">
+        <is>
+          <t>JwtService.java</t>
+        </is>
+      </c>
     </row>
     <row r="25" hidden="1" ht="30" customHeight="1">
       <c r="A25" s="19" t="inlineStr">
@@ -4492,15 +4519,19 @@
       </c>
       <c r="F4" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="G4" s="21" t="inlineStr">
         <is>
-          <t>Applicable to Kryptos due to the multiple cryptographic primitives used across authentication, storage, and signing.</t>
-        </is>
-      </c>
-      <c r="H4" s="21" t="n"/>
+          <t>Crypto primitives in use can be enumerated from code: AES-256/GCM/NoPadding (EncryptionService), Argon2id (SecurityConfig.passwordEncoder), HS256 (JwtService), SHA-256 (AuditService, EncryptionService key derivation), SecureRandom. A formal cryptographic inventory document is pending.</t>
+        </is>
+      </c>
+      <c r="H4" s="21" t="inlineStr">
+        <is>
+          <t>EncryptionService.java; SecurityConfig.java; JwtService.java; AuditService.java</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="45" customHeight="1">
       <c r="A5" s="14" t="inlineStr">
@@ -4734,15 +4765,19 @@
       </c>
       <c r="F11" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G11" s="21" t="inlineStr">
         <is>
-          <t>Applicable to Kryptos due to the risk of timing attacks on hash and token comparisons.</t>
-        </is>
-      </c>
-      <c r="H11" s="21" t="n"/>
+          <t>Cryptographic operations rely on JCE primitives (Cipher AES/GCM, MessageDigest SHA-256), Argon2PasswordEncoder, and io.jsonwebtoken; all are constant-time at the primitive level. Password verification is delegated to Argon2 .matches(), which performs constant-time comparison. No bespoke byte-by-byte secret comparisons exist in the codebase.</t>
+        </is>
+      </c>
+      <c r="H11" s="21" t="inlineStr">
+        <is>
+          <t>EncryptionService; SecurityConfig.passwordEncoder; AuthService.login</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="48" customHeight="1">
       <c r="A12" s="14" t="inlineStr">
@@ -4770,15 +4805,19 @@
       </c>
       <c r="F12" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G12" s="16" t="inlineStr">
         <is>
-          <t>Applicable to Kryptos due to cryptographic failures potentially exposing internals through error responses.</t>
-        </is>
-      </c>
-      <c r="H12" s="16" t="n"/>
+          <t>Cryptographic failures surface via EncryptionException with a generic message ("Failed to decrypt data"); GCM tag verification fails closed (no plaintext returned). No padding-oracle surface exists because AES/GCM does not use block padding.</t>
+        </is>
+      </c>
+      <c r="H12" s="16" t="inlineStr">
+        <is>
+          <t>EncryptionService.decrypt; EncryptionServiceTest.decrypt_shouldThrow…</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="18" customHeight="1">
       <c r="A13" s="13" t="inlineStr">
@@ -4984,15 +5023,19 @@
       </c>
       <c r="F18" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G18" s="16" t="inlineStr">
         <is>
-          <t>Partially applicable to Kryptos because AES-GCM already provides authentication, and Encrypt-then-MAC would only apply if a non-AEAD cipher were introduced.</t>
-        </is>
-      </c>
-      <c r="H18" s="16" t="n"/>
+          <t>AES-GCM is an AEAD mode that internally performs encrypt-then-MAC (ciphertext is computed first, then the GCM authentication tag is computed over IV + AAD + ciphertext). The application never combines encryption + MAC manually.</t>
+        </is>
+      </c>
+      <c r="H18" s="16" t="inlineStr">
+        <is>
+          <t>EncryptionService.encrypt (AES/GCM/NoPadding)</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="20" customHeight="1">
       <c r="A19" s="13" t="inlineStr">
@@ -5158,15 +5201,19 @@
       </c>
       <c r="F23" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G23" s="21" t="inlineStr">
         <is>
-          <t>Applicable to Kryptos due to the derivation of cryptographic keys from user passwords.</t>
-        </is>
-      </c>
-      <c r="H23" s="21" t="n"/>
+          <t>The single password-derived secret in the system (user login password) is processed by Argon2id via Argon2PasswordEncoder.defaultsForSpringSecurity_v5_8 — an approved KDF with built-in key stretching. There is no other password-to-key derivation path.</t>
+        </is>
+      </c>
+      <c r="H23" s="21" t="inlineStr">
+        <is>
+          <t>SecurityConfig.passwordEncoder; AuthService.register/login</t>
+        </is>
+      </c>
     </row>
     <row r="24" ht="18" customHeight="1">
       <c r="A24" s="13" t="inlineStr">
@@ -5252,15 +5299,19 @@
       </c>
       <c r="F26" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G26" s="21" t="inlineStr">
         <is>
-          <t>Applicable to Kryptos due to every cryptographic key being generated from randomness.</t>
-        </is>
-      </c>
-      <c r="H26" s="21" t="n"/>
+          <t>java.security.SecureRandom (used for IVs, secure-wipe random bytes and indirectly via UUID.randomUUID()) is designed to degrade gracefully under heavy demand on the JVM platforms Kryptos targets (Linux /dev/urandom-backed SHA1PRNG / NativePRNG).</t>
+        </is>
+      </c>
+      <c r="H26" s="21" t="inlineStr">
+        <is>
+          <t>EncryptionService.SECURE_RANDOM; FileHandlingService.secureDelete</t>
+        </is>
+      </c>
     </row>
     <row r="27" ht="18" customHeight="1">
       <c r="A27" s="13" t="inlineStr">
@@ -5428,15 +5479,19 @@
       </c>
       <c r="F32" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G32" s="21" t="inlineStr">
         <is>
-          <t>Partially applicable to Kryptos because decrypted credentials exist only during a single request and must be zeroed from memory afterwards.</t>
-        </is>
-      </c>
-      <c r="H32" s="21" t="n"/>
+          <t>Sensitive plaintext lives in memory only for the duration of the operation: passwords are Argon2-hashed before persistence; credential plaintexts are AES-GCM-encrypted before being saved; uploaded byte arrays are zero-filled in CredentialImportExportService.importForOwner finally block; export temp files are 3-pass wiped after the response is written.</t>
+        </is>
+      </c>
+      <c r="H32" s="21" t="inlineStr">
+        <is>
+          <t>AuthService.register; CredentialService.create; CredentialImportExportService.importForOwner; FileHandlingService.secureDelete</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="F1:F32">
@@ -5763,15 +5818,19 @@
       </c>
       <c r="F9" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="G9" s="16" t="inlineStr">
         <is>
-          <t>Applicable to Kryptos due to its public-facing API being accessed over untrusted networks.</t>
-        </is>
-      </c>
-      <c r="H9" s="16" t="n"/>
+          <t>HSTS is set via SecurityConfig (includeSubDomains, max-age=31536000), forcing TLS on browser callers. Actual TLS termination is a reverse-proxy responsibility in the target deployment; documentation of the reverse-proxy contract is pending.</t>
+        </is>
+      </c>
+      <c r="H9" s="16" t="inlineStr">
+        <is>
+          <t>SecurityConfig.httpStrictTransportSecurity</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="51" customHeight="1">
       <c r="A10" s="19" t="inlineStr">
@@ -5889,15 +5948,19 @@
       </c>
       <c r="F13" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="G13" s="21" t="inlineStr">
         <is>
-          <t>Applicable to Kryptos due to the database client needing to verify server identity before sending queries.</t>
-        </is>
-      </c>
-      <c r="H13" s="21" t="n"/>
+          <t>TLS-validating clients are not yet used: the only outbound connection is JDBC → PostgreSQL on the docker-compose private network, currently without sslmode=verify-full. Switching to verified TLS is on the Sprint 3 backlog.</t>
+        </is>
+      </c>
+      <c r="H13" s="21" t="inlineStr">
+        <is>
+          <t>application.properties#spring.datasource.url; docker-compose.yml</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="48" customHeight="1">
       <c r="A14" s="14" t="inlineStr">
@@ -6304,15 +6367,19 @@
       </c>
       <c r="F8" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G8" s="16" t="inlineStr">
         <is>
-          <t>Applicable to Kryptos due to backend communications requiring authenticated service accounts.</t>
-        </is>
-      </c>
-      <c r="H8" s="16" t="n"/>
+          <t>The only backend-to-backend channel is JDBC → PostgreSQL, authenticated with DB_USERNAME + DB_PASSWORD (injected from GitHub repo secrets in CI, from .env locally). No anonymous or shared service connection exists.</t>
+        </is>
+      </c>
+      <c r="H8" s="16" t="inlineStr">
+        <is>
+          <t>application.properties#spring.datasource.{username,password}; docker-compose.yml</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="30" customHeight="1">
       <c r="A9" s="19" t="inlineStr">
@@ -6340,15 +6407,19 @@
       </c>
       <c r="F9" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="G9" s="21" t="inlineStr">
         <is>
-          <t>Applicable to Kryptos due to backend components needing least-privilege credentials.</t>
-        </is>
-      </c>
-      <c r="H9" s="21" t="n"/>
+          <t>PostgreSQL is accessed with a single application-level account that has full ownership of the schema. Splitting into per-role accounts (writer / reader / migration) is on the Sprint 3 backlog.</t>
+        </is>
+      </c>
+      <c r="H9" s="21" t="inlineStr">
+        <is>
+          <t>docker-compose.yml#POSTGRES_USER; application.properties#spring.datasource.username</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="30" customHeight="1">
       <c r="A10" s="14" t="inlineStr">
@@ -6376,15 +6447,19 @@
       </c>
       <c r="F10" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G10" s="16" t="inlineStr">
         <is>
-          <t>Applicable to Kryptos due to the risk posed by shipping default or example credentials.</t>
-        </is>
-      </c>
-      <c r="H10" s="16" t="n"/>
+          <t>No default credentials are baked into the code or images. DB_PASSWORD, JWT_SECRET, ENCRYPTION_SECRET are mandatory env values; JwtService/EncryptionService fail-fast on missing/weak values.</t>
+        </is>
+      </c>
+      <c r="H10" s="16" t="inlineStr">
+        <is>
+          <t>JwtService.getSigningKey; EncryptionService constructor; backend/.env.example</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="30" customHeight="1">
       <c r="A11" s="19" t="inlineStr">
@@ -6412,15 +6487,19 @@
       </c>
       <c r="F11" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G11" s="21" t="inlineStr">
         <is>
-          <t>Applicable to Kryptos due to the need to restrict outbound connections to known trusted hosts.</t>
-        </is>
-      </c>
-      <c r="H11" s="21" t="n"/>
+          <t>The application makes no outbound HTTP/SMB/FTP requests on behalf of users. There is no outbound resource surface that an allowlist would govern; the JDBC URL is the single hard-coded outbound destination.</t>
+        </is>
+      </c>
+      <c r="H11" s="21" t="inlineStr">
+        <is>
+          <t>No outbound HTTP client in backend/src/main/java</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="30" customHeight="1">
       <c r="A12" s="14" t="inlineStr">
@@ -6448,15 +6527,19 @@
       </c>
       <c r="F12" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G12" s="16" t="inlineStr">
         <is>
-          <t>Applicable to Kryptos due to the server requiring an allowlist of permitted outbound destinations.</t>
-        </is>
-      </c>
-      <c r="H12" s="16" t="n"/>
+          <t>Same justification as V13.2.4 — the application does not load data or files from external systems based on user input. The only external endpoint is the JDBC URL, configured via env.</t>
+        </is>
+      </c>
+      <c r="H12" s="16" t="inlineStr">
+        <is>
+          <t>application.properties; SecurityConfig.java</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="30" customHeight="1">
       <c r="A13" s="19" t="inlineStr">
@@ -6538,15 +6621,19 @@
       </c>
       <c r="F15" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="G15" s="16" t="inlineStr">
         <is>
-          <t>Applicable to Kryptos due to the presence of multiple high-value secrets that cannot live in source code.</t>
-        </is>
-      </c>
-      <c r="H15" s="16" t="n"/>
+          <t>Secrets are stored in GitHub Actions repo secrets (CI) and .env files (local dev). GitHub Secrets are encrypted at rest and access-controlled per repo, but adoption of a dedicated secrets manager (e.g., HashiCorp Vault, AWS Secrets Manager) for the production deployment is still planned.</t>
+        </is>
+      </c>
+      <c r="H15" s="16" t="inlineStr">
+        <is>
+          <t>.github/workflows/ci.yml; backend/.env.example</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="30" customHeight="1">
       <c r="A16" s="19" t="inlineStr">
@@ -6574,15 +6661,19 @@
       </c>
       <c r="F16" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G16" s="21" t="inlineStr">
         <is>
-          <t>Applicable to Kryptos due to the sensitivity of the vault secrets accessed by the API.</t>
-        </is>
-      </c>
-      <c r="H16" s="21" t="n"/>
+          <t>GitHub repo secrets are scoped to the repository: only the CI workflow on protected branches can read them, and they are masked from build logs. Local .env files are 0600 and listed in .gitignore.</t>
+        </is>
+      </c>
+      <c r="H16" s="21" t="inlineStr">
+        <is>
+          <t>.github/workflows/ci.yml; backend/.gitignore</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="48" customHeight="1">
       <c r="A17" s="14" t="inlineStr">
@@ -6700,15 +6791,19 @@
       </c>
       <c r="F20" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G20" s="16" t="inlineStr">
         <is>
-          <t>Applicable to Kryptos due to the risk of leaking source-control metadata in production deployments.</t>
-        </is>
-      </c>
-      <c r="H20" s="16" t="n"/>
+          <t>The production image is produced by a multi-stage Dockerfile: the final JRE-only stage copies just the built JAR. No .git, no .svn, no source files are shipped.</t>
+        </is>
+      </c>
+      <c r="H20" s="16" t="inlineStr">
+        <is>
+          <t>backend/Dockerfile</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="30" customHeight="1">
       <c r="A21" s="19" t="inlineStr">
@@ -6856,15 +6951,19 @@
       </c>
       <c r="F24" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G24" s="16" t="inlineStr">
         <is>
-          <t>Applicable to Kryptos due to internal documentation and monitoring endpoints that must not be publicly exposed.</t>
-        </is>
-      </c>
-      <c r="H24" s="16" t="n"/>
+          <t>No documentation or monitoring endpoints are enabled: there is no spring-boot-starter-actuator dependency, no springdoc-openapi dependency, and no Swagger UI bean. The /v3/api-docs/** and /swagger-ui/** SecurityConfig permits resolve to 404 in practice.</t>
+        </is>
+      </c>
+      <c r="H24" s="16" t="inlineStr">
+        <is>
+          <t>backend/pom.xml; SecurityConfig.java</t>
+        </is>
+      </c>
     </row>
     <row r="25" ht="30" customHeight="1">
       <c r="A25" s="19" t="inlineStr">
@@ -6892,15 +6991,19 @@
       </c>
       <c r="F25" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="G25" s="21" t="inlineStr">
         <is>
-          <t>Applicable to Kryptos due to error responses possibly leaking internal system data.</t>
-        </is>
-      </c>
-      <c r="H25" s="21" t="n"/>
+          <t>Spring Boot may emit a Server header by default. Suppressing it via server.server-header= (and verifying via ZAP) is a small Sprint 3 hardening task.</t>
+        </is>
+      </c>
+      <c r="H25" s="21" t="inlineStr">
+        <is>
+          <t>application.properties (no server.server-header configured yet)</t>
+        </is>
+      </c>
     </row>
     <row r="26" ht="30" customHeight="1">
       <c r="A26" s="14" t="inlineStr">
@@ -6928,15 +7031,19 @@
       </c>
       <c r="F26" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G26" s="16" t="inlineStr">
         <is>
-          <t>Applicable to Kryptos due to server-identifying headers enabling fingerprinting.</t>
-        </is>
-      </c>
-      <c r="H26" s="16" t="n"/>
+          <t>The web tier serves only JSON responses generated by controllers; there is no static-file handler registered, no static directory exposed, and no file-extension-based content serving.</t>
+        </is>
+      </c>
+      <c r="H26" s="16" t="inlineStr">
+        <is>
+          <t>KryptosApplication.java; SecurityConfig.java</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="F1:F26"/>
@@ -7754,15 +7861,19 @@
       </c>
       <c r="F5" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="G5" s="44" t="inlineStr">
         <is>
-          <t>Applicable to Kryptos due to potentially resource-demanding operations such as credential import/export, temporary file generation, secure wipe procedures, and audit-related processing. This requirement may be addressed by documenting such operations and by considering controls such as request limits, controlled concurrency, asynchronous processing, or queue-based handling to reduce availability risks.</t>
-        </is>
-      </c>
-      <c r="H5" s="16" t="n"/>
+          <t>Time/resource-intensive operations are identified in code (login lockout window, import/export rate limit, AES-GCM encryption per credential, secure 3-pass wipe). A consolidated documentation entry listing these and their availability protections is pending.</t>
+        </is>
+      </c>
+      <c r="H5" s="16" t="inlineStr">
+        <is>
+          <t>AuthService.java; ImportExportRateLimiter.java; FileHandlingService.java</t>
+        </is>
+      </c>
       <c r="I5" s="47" t="n"/>
     </row>
     <row r="6" ht="30" customHeight="1">
@@ -7957,15 +8068,19 @@
       </c>
       <c r="F11" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G11" s="44" t="inlineStr">
         <is>
-          <t>Highly applicable to Kryptos, especially because the production environment should expose only the functionality strictly necessary for secure operation. This may be addressed by excluding development-only features, test code, sample content, debugging endpoints, and any unnecessary operating system functionality from the production deployment.</t>
-        </is>
-      </c>
-      <c r="H11" s="16" t="n"/>
+          <t>Production build = mvn package output of src/main only. Test code (src/test) is not packaged into the JAR; no sample data is loaded; no debug or developer endpoints are exposed (no actuator dependency).</t>
+        </is>
+      </c>
+      <c r="H11" s="16" t="inlineStr">
+        <is>
+          <t>backend/Dockerfile; backend/pom.xml</t>
+        </is>
+      </c>
       <c r="I11" s="47" t="n"/>
     </row>
     <row r="12" ht="30" customHeight="1">
@@ -8222,15 +8337,19 @@
       </c>
       <c r="F19" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G19" s="44" t="inlineStr">
         <is>
-          <t>Applicable to Kryptos as a general secure coding requirement, especially in authentication, authorization, input validation, and data-processing logic. This requirement may be addressed by enforcing type safety, validating expected data types explicitly, and using strict equality and comparison operations to reduce the risk of type confusion or type juggling vulnerabilities.</t>
-        </is>
-      </c>
-      <c r="H19" s="16" t="n"/>
+          <t>Java enforces static typing at compile time. Equality comparisons use .equals() for objects (username/email comparisons) and primitive == for primitives. No type juggling is possible.</t>
+        </is>
+      </c>
+      <c r="H19" s="16" t="inlineStr">
+        <is>
+          <t>AuthService.login; UserService.findById; all DTO records</t>
+        </is>
+      </c>
       <c r="I19" s="34" t="n"/>
     </row>
     <row r="20" ht="30" customHeight="1">
@@ -8374,15 +8493,19 @@
       </c>
       <c r="F24" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G24" s="45" t="inlineStr">
         <is>
-          <t>Highly applicable to Kryptos, especially in operations involving file handling, temporary file deletion, and access-controlled resources such as vaults and credentials. This requirement may be addressed by ensuring that security-relevant checks and the corresponding actions are performed as closely and atomically as possible, in order to reduce TOCTOU-related risks.</t>
-        </is>
-      </c>
-      <c r="H24" s="21" t="n"/>
+          <t>All check-then-act sequences run inside an @Transactional service method, giving a consistent read-modify-write window (existsByIdAndOwnerId → save inside the same transaction). The file-system check-then-act in FileHandlingService is bounded by a normalised path + CREATE_NEW flag, which fails closed on race.</t>
+        </is>
+      </c>
+      <c r="H24" s="21" t="inlineStr">
+        <is>
+          <t>CredentialService.create; VaultService.delete; FileHandlingService.exportCredentials (CREATE_NEW)</t>
+        </is>
+      </c>
       <c r="I24" s="47" t="n"/>
     </row>
     <row r="25" ht="30" customHeight="1">
@@ -8588,15 +8711,19 @@
       </c>
       <c r="F3" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="G3" s="27" t="inlineStr">
         <is>
-          <t>Highly applicable to Kryptos. Logging should be documented across the application layers, including logged events, formats, storage location, access control, intended use, and retention period.</t>
-        </is>
-      </c>
-      <c r="H3" s="16" t="n"/>
+          <t>The full set of security events is enumerated in AuditAction (LOGIN, LOGIN_FAILED, REGISTER, CREDENTIAL_*, VAULT_*, USER_*, DEVICE_*, EXPORT, IMPORT, SECURE_WIPE*). Logs are written to the audit_logs table via AuditService. A formal logging-inventory document covering Spring access logs, application logs and audit logs is still pending.</t>
+        </is>
+      </c>
+      <c r="H3" s="16" t="inlineStr">
+        <is>
+          <t>AuditAction.java; AuditService.java; application.properties#logging</t>
+        </is>
+      </c>
       <c r="I3" s="34" t="n"/>
     </row>
     <row r="4" ht="18" customHeight="1">
@@ -9894,15 +10021,19 @@
       </c>
       <c r="F3" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G3" s="28" t="inlineStr">
         <is>
-          <t>Applicable to Kryptos due to the processing of API request data and imported files.</t>
-        </is>
-      </c>
-      <c r="H3" s="16" t="n"/>
+          <t>Spring MVC / Jackson decode the HTTP request body into the typed DTO record exactly once. The application performs no manual URL decoding loops or double-decoding of any inbound value.</t>
+        </is>
+      </c>
+      <c r="H3" s="16" t="inlineStr">
+        <is>
+          <t>Spring Boot 3.5 default request pipeline; *Controller.java</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="19" t="inlineStr">
@@ -9930,15 +10061,19 @@
       </c>
       <c r="F4" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G4" s="21" t="inlineStr">
         <is>
-          <t>Applicable to Kryptos due to ensure the backend automatically escapes all outgoing data</t>
-        </is>
-      </c>
-      <c r="H4" s="21" t="n"/>
+          <t>Output JSON is generated by Jackson which encodes/escapes values automatically. Audit-log details are CRLF/control-char-stripped by AuditService.sanitize() before being written.</t>
+        </is>
+      </c>
+      <c r="H4" s="21" t="inlineStr">
+        <is>
+          <t>AuditService.java#sanitize; Spring default ObjectMapper</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="18" customHeight="1">
       <c r="A5" s="13" t="inlineStr">
@@ -10056,15 +10191,19 @@
       </c>
       <c r="F8" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G8" s="16" t="inlineStr">
         <is>
-          <t>Applicable to Kryptos due to the API's continuous generation of dynamic JSON responses; need to enforce safe JSON serialization and avoid manual string concatenation.</t>
-        </is>
-      </c>
-      <c r="H8" s="16" t="n"/>
+          <t>All responses are JSON serialised by Jackson, which encodes special characters in string values (e.g., quotes, backslashes, control chars).</t>
+        </is>
+      </c>
+      <c r="H8" s="16" t="inlineStr">
+        <is>
+          <t>Spring Boot default Jackson MessageConverter</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="30" customHeight="1">
       <c r="A9" s="19" t="inlineStr">
@@ -10092,15 +10231,19 @@
       </c>
       <c r="F9" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G9" s="21" t="inlineStr">
         <is>
-          <t>Applicable to Kryptos due to database interactions; need to strictly enforce parameterized queries or secure ORMs to prevent SQL injection.</t>
-        </is>
-      </c>
-      <c r="H9" s="21" t="n"/>
+          <t>Persistence goes exclusively through Spring Data JPA repositories with derived methods (findAllByOwnerId, existsByIdAndOwnerId, etc.); there is no native SQL / HQL / JPQL string concatenation anywhere in the codebase.</t>
+        </is>
+      </c>
+      <c r="H9" s="21" t="inlineStr">
+        <is>
+          <t>backend/src/main/java/com/kryptos/**/domain/*Repository.java</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="30" customHeight="1">
       <c r="A10" s="14" t="inlineStr">
@@ -10128,15 +10271,19 @@
       </c>
       <c r="F10" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G10" s="16" t="inlineStr">
         <is>
-          <t>Applicable to Kryptos due to OS-level temporary file handling; need to ensure any system calls avoid direct concatenation to prevent command injection.</t>
-        </is>
-      </c>
-      <c r="H10" s="16" t="n"/>
+          <t>No OS command invocation exists: there is zero use of Runtime.exec, ProcessBuilder, or Process. All file operations use java.nio.file (Path/Files) and never shell out.</t>
+        </is>
+      </c>
+      <c r="H10" s="16" t="inlineStr">
+        <is>
+          <t>FileHandlingService.java; grep over backend/src/main</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="30" customHeight="1">
       <c r="A11" s="19" t="inlineStr">
@@ -10260,15 +10407,19 @@
       </c>
       <c r="F14" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G14" s="16" t="inlineStr">
         <is>
-          <t>Applicable to Kryptos due to regex-based input validation; need to ensure special characters are safely escaped to prevent regex injection.</t>
-        </is>
-      </c>
-      <c r="H14" s="16" t="n"/>
+          <t>The only regex literals in the codebase are static and non-user-controlled: [\\x00-\\x1F\\x7F] (sanitization), [A-Za-z0-9]{1,8} (extension allowlist). No regex is composed with user input.</t>
+        </is>
+      </c>
+      <c r="H14" s="16" t="inlineStr">
+        <is>
+          <t>AuditService.sanitize; CredentialImportExportService.safe; FileHandlingService.storeUpload</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="30" customHeight="1">
       <c r="A15" s="19" t="inlineStr">
@@ -10378,15 +10529,19 @@
       </c>
       <c r="F18" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G18" s="21" t="inlineStr">
         <is>
-          <t>Applicable to Kryptos due to backend logic execution; need to strictly avoid dynamic code execution like eval() or sanitize input if unavoidable</t>
-        </is>
-      </c>
-      <c r="H18" s="21" t="n"/>
+          <t>No use of Spring Expression Language with user input. @PreAuthorize expressions are literal strings ("hasRole('USER')" etc.). No reflection-based code execution.</t>
+        </is>
+      </c>
+      <c r="H18" s="21" t="inlineStr">
+        <is>
+          <t>All @PreAuthorize sites in backend/src/main/java/com/kryptos/**/api/</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="30" customHeight="1">
       <c r="A19" s="14" t="inlineStr">
@@ -10414,15 +10569,19 @@
       </c>
       <c r="F19" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G19" s="16" t="inlineStr">
         <is>
-          <t>Applicable to Kryptos due to untrusted input handling; need to sanitize data length and characters before reaching potentially dangerous contexts.</t>
-        </is>
-      </c>
-      <c r="H19" s="16" t="n"/>
+          <t>AuditService.sanitize strips control characters and CRLF before persistence; CredentialImportExportService.safe truncates and strips control chars before writing imported strings to JPA.</t>
+        </is>
+      </c>
+      <c r="H19" s="16" t="inlineStr">
+        <is>
+          <t>AuditService.sanitize; CredentialImportExportService.safe; AuditServiceTest.log_shouldSanitizeDetails</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="30" customHeight="1">
       <c r="A20" s="19" t="inlineStr">
@@ -10514,15 +10673,19 @@
       </c>
       <c r="F22" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G22" s="21" t="inlineStr">
         <is>
-          <t>Applicable to Kryptos due to potential outbound network requests; need to validate URLs against an allowlist to prevent SSRF.</t>
-        </is>
-      </c>
-      <c r="H22" s="21" t="n"/>
+          <t>Kryptos performs no outbound HTTP/URL fetches based on user-supplied data. The application has zero SSRF surface: no HTTP client is instantiated with a user-controlled URL, no URL fields exist in any DTO that are dereferenced server-side.</t>
+        </is>
+      </c>
+      <c r="H22" s="21" t="inlineStr">
+        <is>
+          <t>No RestTemplate / WebClient / HttpClient usage anywhere in backend/src/main/java</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="30" customHeight="1">
       <c r="A23" s="14" t="inlineStr">
@@ -10550,15 +10713,19 @@
       </c>
       <c r="F23" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G23" s="16" t="inlineStr">
         <is>
-          <t>Applicable to Kryptos due to dynamic file or message generation; need to prevent template injection by strictly sanitizing untrusted input in templates.</t>
-        </is>
-      </c>
-      <c r="H23" s="16" t="n"/>
+          <t>Kryptos has no template engine. There is no Thymeleaf, Freemarker, Velocity, Mustache, or any other templating library declared in pom.xml. Responses are JSON, generated by Jackson.</t>
+        </is>
+      </c>
+      <c r="H23" s="16" t="inlineStr">
+        <is>
+          <t>backend/pom.xml (no template engine dependencies)</t>
+        </is>
+      </c>
     </row>
     <row r="24" ht="30" customHeight="1">
       <c r="A24" s="19" t="inlineStr">
@@ -10586,15 +10753,19 @@
       </c>
       <c r="F24" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G24" s="21" t="inlineStr">
         <is>
-          <t>Still unsure what programming language we are going to use</t>
-        </is>
-      </c>
-      <c r="H24" s="21" t="n"/>
+          <t>No JNDI lookup paths exist in the codebase. No InitialContext / Context.lookup() calls. Spring Boot is configured with a direct JDBC DataSource (no JNDI DataSource lookup).</t>
+        </is>
+      </c>
+      <c r="H24" s="21" t="inlineStr">
+        <is>
+          <t>application.properties#spring.datasource.url; SecurityConfig.java</t>
+        </is>
+      </c>
     </row>
     <row r="25" ht="30" customHeight="1">
       <c r="A25" s="14" t="inlineStr">
@@ -10654,15 +10825,19 @@
       </c>
       <c r="F26" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G26" s="28" t="inlineStr">
         <is>
-          <t>Applicable to Kryptos due to backend string formatting, we must strictly avoid user-controllable format strings.</t>
-        </is>
-      </c>
-      <c r="H26" s="21" t="n"/>
+          <t>Java does not expose C-style format-string vulnerabilities (compiler enforces type safety on String.format placeholders). All String.format calls in the codebase use static literal format strings.</t>
+        </is>
+      </c>
+      <c r="H26" s="21" t="inlineStr">
+        <is>
+          <t>AuditService.java; FileHandlingService.java</t>
+        </is>
+      </c>
     </row>
     <row r="27" ht="30" customHeight="1">
       <c r="A27" s="14" t="inlineStr">
@@ -10722,15 +10897,19 @@
       </c>
       <c r="F28" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G28" s="21" t="inlineStr">
         <is>
-          <t>Applicable to Kryptos due to regex-based input validation; need to ensure patterns are safe from ReDoS</t>
-        </is>
-      </c>
-      <c r="H28" s="21" t="n"/>
+          <t>The two regex literals in use are ReDoS-safe: [\\x00-\\x1F\\x7F] (single character class) and [A-Za-z0-9]{1,8} (bounded, no nested quantifiers, no alternation). User input is matched, never used to build a pattern.</t>
+        </is>
+      </c>
+      <c r="H28" s="21" t="inlineStr">
+        <is>
+          <t>AuditService.sanitize; FileHandlingService.storeUpload</t>
+        </is>
+      </c>
     </row>
     <row r="29" ht="18" customHeight="1">
       <c r="A29" s="13" t="inlineStr">
@@ -10776,15 +10955,19 @@
       </c>
       <c r="F30" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G30" s="16" t="inlineStr">
         <is>
-          <t>Applicable to Kryptos due to data processing; need to ensure the backend implementation provides native protection against buffer overflows.</t>
-        </is>
-      </c>
-      <c r="H30" s="16" t="n"/>
+          <t>Java is a memory-safe language: no pointer arithmetic, no manual buffer management, no JNI / Unsafe usage. The codebase exclusively uses Java collections and java.nio buffers.</t>
+        </is>
+      </c>
+      <c r="H30" s="16" t="inlineStr">
+        <is>
+          <t>Language-level guarantee; backend/src/main</t>
+        </is>
+      </c>
     </row>
     <row r="31" ht="30" customHeight="1">
       <c r="A31" s="19" t="inlineStr">
@@ -10812,15 +10995,19 @@
       </c>
       <c r="F31" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G31" s="21" t="inlineStr">
         <is>
-          <t>Applicable to Kryptos due to numeric data handling; need to implement range and sign validation to prevent integer overflow vulnerabilities.</t>
-        </is>
-      </c>
-      <c r="H31" s="21" t="n"/>
+          <t>DTOs enforce input ranges via @Size on length-bounded fields (username, email, password, vault names). File-size and record-count limits use long arithmetic with explicit bounds (5 MiB cap, 50 000 lines). Java overflow semantics are well defined.</t>
+        </is>
+      </c>
+      <c r="H31" s="21" t="inlineStr">
+        <is>
+          <t>RegisterRequest.java; CreateVaultRequest.java; FileHandlingService.java</t>
+        </is>
+      </c>
     </row>
     <row r="32" ht="30" customHeight="1">
       <c r="A32" s="14" t="inlineStr">
@@ -10930,15 +11117,19 @@
       </c>
       <c r="F35" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G35" s="21" t="inlineStr">
         <is>
-          <t>Applicable to Kryptos due to JSON deserialization; need to enforce strict type checking and use safe deserialization libraries for untrusted data.</t>
-        </is>
-      </c>
-      <c r="H35" s="21" t="n"/>
+          <t>Jackson deserialisation uses an explicit target type (ObjectMapper.readValue(..., CredentialExportRecord.class)); polymorphic typing is not enabled, so attacker cannot influence the class instantiated. Java built-in serialization is not used anywhere.</t>
+        </is>
+      </c>
+      <c r="H35" s="21" t="inlineStr">
+        <is>
+          <t>CredentialImportExportService.java#importForOwner</t>
+        </is>
+      </c>
     </row>
     <row r="36" ht="30" customHeight="1">
       <c r="A36" s="14" t="inlineStr">
@@ -10966,15 +11157,19 @@
       </c>
       <c r="F36" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G36" s="16" t="inlineStr">
         <is>
-          <t>Applicable to Kryptos due to the use of multiple data parsers; need to ensure consistent parsing behavior across all components to avoid interoperability flaws.</t>
-        </is>
-      </c>
-      <c r="H36" s="16" t="n"/>
+          <t>Only one parser (Jackson) is in use for the only structured data format (JSON). There is no XML, YAML, or alternative JSON parser, so parser-divergence vulnerabilities are not exposed.</t>
+        </is>
+      </c>
+      <c r="H36" s="16" t="inlineStr">
+        <is>
+          <t>backend/pom.xml; CredentialImportExportService.java</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <conditionalFormatting sqref="F2:F36">
@@ -11368,15 +11563,19 @@
       </c>
       <c r="F11" s="18" t="inlineStr">
         <is>
-          <t>Not Applicable</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G11" s="16" t="inlineStr">
         <is>
-          <t>Kryptos exposes a stateless REST API. There are no multi-step server-side business flows whose order needs enforcing.</t>
-        </is>
-      </c>
-      <c r="H11" s="16" t="n"/>
+          <t>Kryptos exposes a stateless REST API; every authenticated request is independently authorized via @PreAuthorize and ownership checks. There are no multi-step server-side flows whose sequence could be bypassed, so step-skipping is not exploitable.</t>
+        </is>
+      </c>
+      <c r="H11" s="16" t="inlineStr">
+        <is>
+          <t>All controllers under backend/src/main/java/com/kryptos/**/api/</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="30" customHeight="1">
       <c r="A12" s="19" t="inlineStr">
@@ -11606,15 +11805,19 @@
       </c>
       <c r="F18" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G18" s="21" t="inlineStr">
         <is>
-          <t>Applicable to Kryptos due to sensitive business logic flows; need to enforce timing-based controls to prevent excessively rapid transaction submissions.</t>
-        </is>
-      </c>
-      <c r="H18" s="21" t="n"/>
+          <t>Anti-automation realised through ImportExportRateLimiter (5 req/min/principal on import and export) and AuthService (5 login attempts/min/principal → 15 min lockout). Both implement the "no rapid submissions" intent of the requirement.</t>
+        </is>
+      </c>
+      <c r="H18" s="21" t="inlineStr">
+        <is>
+          <t>AuthService.java; ImportExportRateLimiter.java; ImportExportRateLimiterTest</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <conditionalFormatting sqref="F2:F18">
@@ -13018,15 +13221,19 @@
       </c>
       <c r="F5" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G5" s="16" t="inlineStr">
         <is>
-          <t>Applicable to Kryptos due to potential deployment behind proxies/load balancers; need to ensure user-supplied headers cannot override system-set headers.</t>
-        </is>
-      </c>
-      <c r="H5" s="16" t="n"/>
+          <t>The application reads identity exclusively from @AuthenticationPrincipal (set by JwtAuthFilter after verifying the Authorization Bearer token). It does not read X-Forwarded-User / X-User-Id / X-Real-IP or any intermediary-set identity header. Spring Boot default server.forward-headers-strategy is NONE.</t>
+        </is>
+      </c>
+      <c r="H5" s="16" t="inlineStr">
+        <is>
+          <t>JwtAuthFilter.java; SecurityConfig.java; all controllers</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="30" customHeight="1">
       <c r="A6" s="19" t="inlineStr">
@@ -13148,15 +13355,19 @@
       </c>
       <c r="F9" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G9" s="16" t="inlineStr">
         <is>
-          <t>Applicable to Kryptos due to sensitive vault and credential data; need to enforce strict JWT-based authentication and authorization for every API endpoint.</t>
-        </is>
-      </c>
-      <c r="H9" s="16" t="n"/>
+          <t>HTTP message boundary parsing is delegated to the Spring Boot embedded Tomcat connector, which correctly handles Content-Length and Transfer-Encoding per RFC 7230 and rejects ambiguous messages by default.</t>
+        </is>
+      </c>
+      <c r="H9" s="16" t="inlineStr">
+        <is>
+          <t>Spring Boot 3.5 embedded Tomcat defaults</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="30" customHeight="1">
       <c r="A10" s="19" t="inlineStr">
@@ -13184,15 +13395,19 @@
       </c>
       <c r="F10" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G10" s="21" t="inlineStr">
         <is>
-          <t>Applicable to Kryptos due to multi-tenant vault management; need to implement ownership checks to ensure users only access their own credentials.</t>
-        </is>
-      </c>
-      <c r="H10" s="21" t="n"/>
+          <t>Responses are produced by Spring MVC; Content-Length is set automatically to match the serialized body length. No manual Content-Length writes anywhere in the code.</t>
+        </is>
+      </c>
+      <c r="H10" s="21" t="inlineStr">
+        <is>
+          <t>Spring MVC default ResponseBodyEmitter / HttpMessageConverter behaviour</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="30" customHeight="1">
       <c r="A11" s="14" t="inlineStr">
@@ -13220,15 +13435,19 @@
       </c>
       <c r="F11" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G11" s="16" t="inlineStr">
         <is>
-          <t>Applicable to Kryptos due to entity update operations; need to use Data Transfer Objects (DTOs) to prevent users from updating fields they shouldn't.</t>
-        </is>
-      </c>
-      <c r="H11" s="16" t="n"/>
+          <t>Tomcat HTTP/2 connector rejects connection-specific header fields per RFC 7540 §8.1.2.2 by default. Application does not synthesise such headers anywhere.</t>
+        </is>
+      </c>
+      <c r="H11" s="16" t="inlineStr">
+        <is>
+          <t>Embedded Tomcat HTTP/2 defaults</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="30" customHeight="1">
       <c r="A12" s="19" t="inlineStr">
@@ -13256,15 +13475,19 @@
       </c>
       <c r="F12" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G12" s="21" t="inlineStr">
         <is>
-          <t>Applicable to Kryptos due to strict JSON requirements; need to configure the API to reject any requests with unsupported Content-Types.</t>
-        </is>
-      </c>
-      <c r="H12" s="21" t="n"/>
+          <t>CR / LF in header names or values are rejected by Tomcat at the HTTP-parser level. Application does not assemble headers from user input — the only response headers come from controller code with static names + bounded values (Content-Type, Content-Disposition, Cache-Control, X-Content-Type-Options).</t>
+        </is>
+      </c>
+      <c r="H12" s="21" t="inlineStr">
+        <is>
+          <t>ImportExportController.exportCredentials; SecurityConfig.headers(...)</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="30" customHeight="1">
       <c r="A13" s="14" t="inlineStr">
@@ -13292,15 +13515,19 @@
       </c>
       <c r="F13" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G13" s="28" t="inlineStr">
         <is>
-          <t>Applicable to Kryptos due to error response handling; need to implement global exception handlers to strip stack traces and internal DB details from API responses.</t>
-        </is>
-      </c>
-      <c r="H13" s="16" t="n"/>
+          <t>The backend does not build or send outbound HTTP requests on behalf of users. There is no RestTemplate / WebClient / HttpClient usage, so URI- or header-injection on outbound calls is not reachable.</t>
+        </is>
+      </c>
+      <c r="H13" s="16" t="inlineStr">
+        <is>
+          <t>No outbound HTTP client in backend/src/main/java</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="18" customHeight="1">
       <c r="A14" s="13" t="inlineStr">
@@ -13796,15 +14023,19 @@
       </c>
       <c r="F7" s="18" t="inlineStr">
         <is>
-          <t>Not Applicable</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Kryptos does not accept compressed archives. Only single-file .kvault uploads (newline-delimited encrypted records) are processed.</t>
-        </is>
-      </c>
-      <c r="H7" s="16" t="n"/>
+          <t>Kryptos accepts only newline-delimited .kvault import files; no compressed archives (zip, gz, tar, etc.) are decompressed. The compression-bomb attack surface is therefore absent. Hard caps remain in place: 5 MiB payload (HTTP 413) and 50 000 lines.</t>
+        </is>
+      </c>
+      <c r="H7" s="16" t="inlineStr">
+        <is>
+          <t>ImportExportController#importCredentials; FileHandlingService#importCredentials</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="30" customHeight="1">
       <c r="A8" s="19" t="inlineStr">
@@ -13832,15 +14063,19 @@
       </c>
       <c r="F8" s="18" t="inlineStr">
         <is>
-          <t>Not Applicable</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G8" s="21" t="inlineStr">
         <is>
-          <t>Files are not retained per user. Uploads are stored briefly in the per-process temp directory, parsed, and immediately securely wiped; exports are streamed once and then wiped. No persistent user file storage.</t>
-        </is>
-      </c>
-      <c r="H8" s="21" t="n"/>
+          <t>Files are never retained per user: every upload is parsed and securely wiped within the same request, every export streams a freshly built temp file that is wiped immediately after the response body is written. ImportExportRateLimiter caps both endpoints at 5 requests/min/principal → 429.</t>
+        </is>
+      </c>
+      <c r="H8" s="21" t="inlineStr">
+        <is>
+          <t>CredentialImportExportService#importForOwner/exportForOwner; FileHandlingService#secureDelete; ImportExportRateLimiter</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="30" customHeight="1">
       <c r="A9" s="14" t="inlineStr">
@@ -13868,15 +14103,19 @@
       </c>
       <c r="F9" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>This prevents Kryptos from being exposed to path traversal or unauthorized file access attacks that could occur if malicious symlinks inside uploaded archives are processed.</t>
-        </is>
-      </c>
-      <c r="H9" s="16" t="n"/>
+          <t>Compressed archives are not accepted by any endpoint (see V5.2.3); symlink-in-archive cannot be reached because no decompression is performed.</t>
+        </is>
+      </c>
+      <c r="H9" s="16" t="inlineStr">
+        <is>
+          <t>ImportExportController; FileHandlingService</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="30" customHeight="1">
       <c r="A10" s="19" t="inlineStr">
@@ -14033,15 +14272,19 @@
       </c>
       <c r="F14" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Ignoring user-supplied paths during file processing in Kryptos prevents zip slip attacks that could overwrite or access unintended files on the server.</t>
-        </is>
-      </c>
-      <c r="H14" s="16" t="n"/>
+          <t>No server-side decompression occurs. Zip-slip / path-traversal-via-archive is not exposed. The single path-traversal mitigation on the upload path is verifyWithinTempDir(), enforced on every read/write.</t>
+        </is>
+      </c>
+      <c r="H14" s="16" t="inlineStr">
+        <is>
+          <t>FileHandlingService#verifyWithinTempDir; FileHandlingServiceTest.secureDelete_refusesPathOutsideTempDir</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="18" customHeight="1">
       <c r="A15" s="13" t="inlineStr">
@@ -14305,15 +14548,19 @@
       </c>
       <c r="F3" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Define and apply protections like rate limiting and anti-automation to stop brute force and credential stuffing attacks without enabling denial of service through account lockout.</t>
-        </is>
-      </c>
-      <c r="H3" s="16" t="n"/>
+          <t>Rate-limiting / anti-automation controls are implemented (5 attempts/15-min lockout on login; 5 req/min on import/export). A formal "authentication anti-automation controls" documentation entry in the security baseline is still pending.</t>
+        </is>
+      </c>
+      <c r="H3" s="16" t="inlineStr">
+        <is>
+          <t>AuthService.java; ImportExportRateLimiter.java</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="19" t="inlineStr">
@@ -14377,15 +14624,19 @@
       </c>
       <c r="F5" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Documents all authentication methods in Kryptos with consistent security controls and strength, preventing weaker pathways from undermining overall authentication security.</t>
-        </is>
-      </c>
-      <c r="H5" s="16" t="n"/>
+          <t>Kryptos exposes a single authentication pathway (username/email + password → JWT issuance at POST /api/auth/login). No alternative authentication routes (SSO, certificate, API key) exist, so multi-pathway consistency is trivially satisfied.</t>
+        </is>
+      </c>
+      <c r="H5" s="16" t="inlineStr">
+        <is>
+          <t>AuthController.java; AuthService.login</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="18" customHeight="1">
       <c r="A6" s="13" t="inlineStr">
@@ -14615,15 +14866,15 @@
       </c>
       <c r="F12" s="18" t="inlineStr">
         <is>
-          <t>Not Applicable</t>
+          <t>Not Started</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Backend-only project; password masking (type=password) is a frontend concern and out of scope.</t>
-        </is>
-      </c>
-      <c r="H12" s="21" t="n"/>
+          <t>Backend-only project; UI-side password masking (type=password) requires a frontend. This will be addressed when a client UI is integrated.</t>
+        </is>
+      </c>
+      <c r="H12" s="21" t="inlineStr"/>
     </row>
     <row r="13" ht="30" customHeight="1">
       <c r="A13" s="14" t="inlineStr">
@@ -14651,15 +14902,15 @@
       </c>
       <c r="F13" s="18" t="inlineStr">
         <is>
-          <t>Not Applicable</t>
+          <t>Not Started</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Backend-only project; paste / password-manager support is a frontend concern.</t>
-        </is>
-      </c>
-      <c r="H13" s="16" t="n"/>
+          <t>Backend-only project; paste / browser password manager support is a frontend concern. Will be revisited when the UI is in scope.</t>
+        </is>
+      </c>
+      <c r="H13" s="16" t="inlineStr"/>
     </row>
     <row r="14" ht="30" customHeight="1">
       <c r="A14" s="19" t="inlineStr">
@@ -15009,15 +15260,19 @@
       </c>
       <c r="F23" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>Prevents  having hidden or weaker authentication paths by ensuring all methods are documented and enforce consistent security controls.</t>
-        </is>
-      </c>
-      <c r="H23" s="21" t="n"/>
+          <t>Same as V6.1.3 — exactly one authentication pathway exists, so there are no undocumented alternatives and security strength is enforced consistently (Argon2 + 5/15 lockout + JWT issuance).</t>
+        </is>
+      </c>
+      <c r="H23" s="21" t="inlineStr">
+        <is>
+          <t>AuthController.java</t>
+        </is>
+      </c>
     </row>
     <row r="24" ht="30" customHeight="1">
       <c r="A24" s="14" t="inlineStr">
@@ -15203,15 +15458,19 @@
       </c>
       <c r="F29" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G29" s="16" t="inlineStr">
         <is>
-          <t>Verify that system generated initial passwords or activation codes are securely randomly generated, follow the existing password policy, and expire after a short period of time or after they are initially used. These initial secrets must not be permitted to become the long term password.</t>
-        </is>
-      </c>
-      <c r="H29" s="16" t="n"/>
+          <t>Kryptos does not generate initial passwords or activation codes; users set their own password at registration (validated via @Size(min=12)). The attack surface for predictable system-generated credentials is absent.</t>
+        </is>
+      </c>
+      <c r="H29" s="16" t="inlineStr">
+        <is>
+          <t>AuthService.register; RegisterRequest.java</t>
+        </is>
+      </c>
     </row>
     <row r="30" ht="30" customHeight="1">
       <c r="A30" s="19" t="inlineStr">
@@ -15239,15 +15498,19 @@
       </c>
       <c r="F30" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>Eliminates weak recovery mechanisms, preventing attackers from exploiting easily guessable password hints or security questions.</t>
-        </is>
-      </c>
-      <c r="H30" s="21" t="n"/>
+          <t>No password hints, security questions, or knowledge-based authentication exist in any DTO, service, or endpoint. Password reset (when added) will follow ASVS guidance.</t>
+        </is>
+      </c>
+      <c r="H30" s="21" t="inlineStr">
+        <is>
+          <t>No such feature in backend/src/main/java</t>
+        </is>
+      </c>
     </row>
     <row r="31" ht="30" customHeight="1">
       <c r="A31" s="14" t="inlineStr">
@@ -16183,15 +16446,19 @@
       </c>
       <c r="F3" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Applicable, since Kryptos manages authenticated sessions for access to sensitive credential data, requiring clearly defined and justified session timeout policies.</t>
-        </is>
-      </c>
-      <c r="H3" s="16" t="n"/>
+          <t>Session lifetime is configured via JWT_EXPIRATION (default 3600000 ms = 1 h, documented in backend/.env.example). Formal documentation of the rationale and combined-controls analysis is pending.</t>
+        </is>
+      </c>
+      <c r="H3" s="16" t="inlineStr">
+        <is>
+          <t>application.properties#jwt.expiration; backend/.env.example</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="19" t="inlineStr">
@@ -16381,15 +16648,19 @@
       </c>
       <c r="F9" s="18" t="inlineStr">
         <is>
-          <t>Not Applicable</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Kryptos uses self-contained tokens (JWT/HS256), not opaque reference tokens.</t>
-        </is>
-      </c>
-      <c r="H9" s="16" t="n"/>
+          <t>Kryptos uses self-contained JWTs signed with HS256, not opaque reference tokens. The token integrity is guaranteed by the 256-bit HMAC signature (entropy ≥128 bits enforced at startup by JwtService.getSigningKey, which rejects secrets shorter than 32 bytes).</t>
+        </is>
+      </c>
+      <c r="H9" s="16" t="inlineStr">
+        <is>
+          <t>JwtService.java; JwtServiceTest.constructor_shouldThrow_whenSecretIsTooShort</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="30" customHeight="1">
       <c r="A10" s="19" t="inlineStr">
@@ -16908,15 +17179,19 @@
       </c>
       <c r="F26" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>Ensures correctenforcing of session expiration and re-authentication across IdP and RP interactions, preventing users from remaining authenticated beyond intended security limits.</t>
-        </is>
-      </c>
-      <c r="H26" s="21" t="n"/>
+          <t>A session (JWT) is only issued in response to an explicit POST /api/auth/login with valid credentials supplied by the user. There is no implicit / silent session creation path.</t>
+        </is>
+      </c>
+      <c r="H26" s="21" t="inlineStr">
+        <is>
+          <t>AuthController.login; AuthService.login</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <conditionalFormatting sqref="F2:F26">
@@ -17046,15 +17321,19 @@
       </c>
       <c r="F3" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Applicable to Kryptos since it uses role-based access and handles sensitive credential data, requiring clearly defined authorization rules for functions and data access based on permissions and resource attributes.</t>
-        </is>
-      </c>
-      <c r="H3" s="16" t="n"/>
+          <t>Authorization rules are implemented via @PreAuthorize on every controller method (function-level) and ownership checks in services (data-level). A consolidated authorization documentation artefact mapping endpoints to roles and ownership rules is still pending.</t>
+        </is>
+      </c>
+      <c r="H3" s="16" t="inlineStr">
+        <is>
+          <t>All controllers; Sprint1/ThreatIdentification.md</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="19" t="inlineStr">
@@ -17082,15 +17361,19 @@
       </c>
       <c r="F4" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Applicable to Kryptos as it manages sensitive credential data where certain fields may require restricted read/write access depending on user roles and resource attributes.</t>
-        </is>
-      </c>
-      <c r="H4" s="21" t="n"/>
+          <t>Field-level access is implemented via response DTOs that explicitly omit sensitive fields (CredentialResponse excludes encryptedPassword, UserResponse excludes password hash). Formal field-level access matrix documentation is pending.</t>
+        </is>
+      </c>
+      <c r="H4" s="21" t="inlineStr">
+        <is>
+          <t>CredentialResponse.java; UserResponse.java</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="30" customHeight="1">
       <c r="A5" s="14" t="inlineStr">
@@ -17405,15 +17688,19 @@
       </c>
       <c r="F14" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Applicable, as Kryptos relies on role-based access and sensitive credential data, requiring immediate enforcement of permission changes to prevent unauthorized actions.</t>
-        </is>
-      </c>
-      <c r="H14" s="21" t="n"/>
+          <t>Authorization decisions read claims from the JWT, so changes (e.g., role demotion) only propagate after the token expires. The maximum delay equals JWT_EXPIRATION (1 h by default); documentation of this delay window is pending.</t>
+        </is>
+      </c>
+      <c r="H14" s="21" t="inlineStr">
+        <is>
+          <t>JwtService.generateToken; UserService.updateUserRole; application.properties#jwt.expiration</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="30" customHeight="1">
       <c r="A15" s="14" t="inlineStr">
@@ -17441,15 +17728,19 @@
       </c>
       <c r="F15" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Applicable, since Kryptos exposes a REST API where access to credentials and vaults must always be enforced based on the requesting user’s permissions rather than intermediary services.</t>
-        </is>
-      </c>
-      <c r="H15" s="16" t="n"/>
+          <t>Object access is always decided on the originating subject's permissions: services read the authenticated user via @AuthenticationPrincipal KryptosUserDetails or SecurityContextHolder and pass ownerId into every repository query. No service acts on behalf of another principal.</t>
+        </is>
+      </c>
+      <c r="H15" s="16" t="inlineStr">
+        <is>
+          <t>All controllers; all services</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="18" customHeight="1">
       <c r="A16" s="13" t="inlineStr">

</xml_diff>